<commit_message>
Update World Cup live data
</commit_message>
<xml_diff>
--- a/worldcup-schedule/output/worldcup_2026_schedule.xlsx
+++ b/worldcup-schedule/output/worldcup_2026_schedule.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="完整赛程" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="重点比赛" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="小组积分榜" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="最佳小组第三" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="淘汰赛对阵" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="比赛结果" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="完整赛程" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="重点比赛" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="小组积分榜" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="最佳小组第三" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="淘汰赛对阵" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="比赛结果" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="使用说明" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'完整赛程'!$A$1:$V$105</definedName>
@@ -642,7 +642,7 @@
     <col width="23" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="39" customWidth="1" min="6" max="6"/>
+    <col width="38" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
     <col width="25" customWidth="1" min="8" max="8"/>
     <col width="43" customWidth="1" min="9" max="9"/>
@@ -654,9 +654,9 @@
     <col width="9" customWidth="1" min="15" max="15"/>
     <col width="9" customWidth="1" min="16" max="16"/>
     <col width="9" customWidth="1" min="17" max="17"/>
-    <col width="9" customWidth="1" min="18" max="18"/>
+    <col width="13" customWidth="1" min="18" max="18"/>
     <col width="9" customWidth="1" min="19" max="19"/>
-    <col width="27" customWidth="1" min="20" max="20"/>
+    <col width="22" customWidth="1" min="20" max="20"/>
     <col width="9" customWidth="1" min="21" max="21"/>
     <col width="9" customWidth="1" min="22" max="22"/>
   </cols>
@@ -839,21 +839,33 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
-        </is>
-      </c>
-      <c r="O2" s="2" t="inlineStr"/>
-      <c r="P2" s="2" t="inlineStr"/>
+          <t>已结束</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>90+8</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
       <c r="Q2" s="2" t="inlineStr"/>
-      <c r="R2" s="2" t="inlineStr"/>
+      <c r="R2" s="2" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
       <c r="S2" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="T2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U2" s="2" t="inlineStr"/>
@@ -889,7 +901,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>South Korea vs Czech Republic</t>
+          <t>South Korea vs Czechia</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -929,21 +941,33 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
-        </is>
-      </c>
-      <c r="O3" s="2" t="inlineStr"/>
-      <c r="P3" s="2" t="inlineStr"/>
+          <t>已结束</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>90+7</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
       <c r="Q3" s="2" t="inlineStr"/>
-      <c r="R3" s="2" t="inlineStr"/>
+      <c r="R3" s="2" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr"/>
@@ -979,7 +1003,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Canada vs Bosnia and Herzegovina</t>
+          <t>Canada vs Bosnia &amp; Herzegovina</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -1019,21 +1043,29 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
-        </is>
-      </c>
-      <c r="O4" s="2" t="inlineStr"/>
-      <c r="P4" s="2" t="inlineStr"/>
+          <t>已结束</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>90+6</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
       <c r="Q4" s="2" t="inlineStr"/>
       <c r="R4" s="2" t="inlineStr"/>
       <c r="S4" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="T4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U4" s="2" t="inlineStr"/>
@@ -1069,7 +1101,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>United States vs Paraguay</t>
+          <t>USA vs Paraguay</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -1109,21 +1141,31 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
-        </is>
-      </c>
-      <c r="O5" s="2" t="inlineStr"/>
-      <c r="P5" s="2" t="inlineStr"/>
+          <t>已结束</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="n">
+        <v>90</v>
+      </c>
+      <c r="P5" s="2" t="inlineStr">
+        <is>
+          <t>4-1</t>
+        </is>
+      </c>
       <c r="Q5" s="2" t="inlineStr"/>
-      <c r="R5" s="2" t="inlineStr"/>
+      <c r="R5" s="2" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
       <c r="S5" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="T5" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U5" s="2" t="inlineStr"/>
@@ -1213,7 +1255,7 @@
       </c>
       <c r="T6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U6" s="2" t="inlineStr"/>
@@ -1303,7 +1345,7 @@
       </c>
       <c r="T7" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U7" s="2" t="inlineStr"/>
@@ -1393,7 +1435,7 @@
       </c>
       <c r="T8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U8" s="2" t="inlineStr"/>
@@ -1429,7 +1471,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Australia vs Turkey</t>
+          <t>Australia vs Türkiye</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -1483,7 +1525,7 @@
       </c>
       <c r="T9" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U9" s="2" t="inlineStr"/>
@@ -1573,7 +1615,7 @@
       </c>
       <c r="T10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U10" s="2" t="inlineStr"/>
@@ -1663,7 +1705,7 @@
       </c>
       <c r="T11" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U11" s="2" t="inlineStr"/>
@@ -1753,7 +1795,7 @@
       </c>
       <c r="T12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U12" s="2" t="inlineStr"/>
@@ -1843,7 +1885,7 @@
       </c>
       <c r="T13" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U13" s="2" t="inlineStr"/>
@@ -1879,7 +1921,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Spain vs Cape Verde</t>
+          <t>Spain vs Cape Verde Islands</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -1933,7 +1975,7 @@
       </c>
       <c r="T14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U14" s="2" t="inlineStr"/>
@@ -2023,7 +2065,7 @@
       </c>
       <c r="T15" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U15" s="2" t="inlineStr"/>
@@ -2113,7 +2155,7 @@
       </c>
       <c r="T16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U16" s="2" t="inlineStr"/>
@@ -2203,7 +2245,7 @@
       </c>
       <c r="T17" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U17" s="2" t="inlineStr"/>
@@ -2293,7 +2335,7 @@
       </c>
       <c r="T18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U18" s="2" t="inlineStr"/>
@@ -2383,7 +2425,7 @@
       </c>
       <c r="T19" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U19" s="2" t="inlineStr"/>
@@ -2473,7 +2515,7 @@
       </c>
       <c r="T20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U20" s="2" t="inlineStr"/>
@@ -2563,7 +2605,7 @@
       </c>
       <c r="T21" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U21" s="2" t="inlineStr"/>
@@ -2599,7 +2641,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Portugal vs DR Congo</t>
+          <t>Portugal vs Congo DR</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -2653,7 +2695,7 @@
       </c>
       <c r="T22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U22" s="2" t="inlineStr"/>
@@ -2743,7 +2785,7 @@
       </c>
       <c r="T23" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U23" s="2" t="inlineStr"/>
@@ -2833,7 +2875,7 @@
       </c>
       <c r="T24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U24" s="2" t="inlineStr"/>
@@ -2923,7 +2965,7 @@
       </c>
       <c r="T25" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U25" s="2" t="inlineStr"/>
@@ -2959,7 +3001,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Czech Republic vs South Africa</t>
+          <t>Czechia vs South Africa</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -3013,7 +3055,7 @@
       </c>
       <c r="T26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U26" s="2" t="inlineStr"/>
@@ -3049,7 +3091,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Switzerland vs Bosnia and Herzegovina</t>
+          <t>Switzerland vs Bosnia &amp; Herzegovina</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -3103,7 +3145,7 @@
       </c>
       <c r="T27" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U27" s="2" t="inlineStr"/>
@@ -3193,7 +3235,7 @@
       </c>
       <c r="T28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U28" s="2" t="inlineStr"/>
@@ -3283,7 +3325,7 @@
       </c>
       <c r="T29" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U29" s="2" t="inlineStr"/>
@@ -3319,7 +3361,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>United States vs Australia</t>
+          <t>USA vs Australia</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -3373,7 +3415,7 @@
       </c>
       <c r="T30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U30" s="2" t="inlineStr"/>
@@ -3463,7 +3505,7 @@
       </c>
       <c r="T31" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U31" s="2" t="inlineStr"/>
@@ -3553,7 +3595,7 @@
       </c>
       <c r="T32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U32" s="2" t="inlineStr"/>
@@ -3589,7 +3631,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Turkey vs Paraguay</t>
+          <t>Türkiye vs Paraguay</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -3643,7 +3685,7 @@
       </c>
       <c r="T33" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U33" s="2" t="inlineStr"/>
@@ -3733,7 +3775,7 @@
       </c>
       <c r="T34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U34" s="2" t="inlineStr"/>
@@ -3823,7 +3865,7 @@
       </c>
       <c r="T35" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U35" s="2" t="inlineStr"/>
@@ -3913,7 +3955,7 @@
       </c>
       <c r="T36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U36" s="2" t="inlineStr"/>
@@ -4003,7 +4045,7 @@
       </c>
       <c r="T37" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U37" s="2" t="inlineStr"/>
@@ -4093,7 +4135,7 @@
       </c>
       <c r="T38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U38" s="2" t="inlineStr"/>
@@ -4183,7 +4225,7 @@
       </c>
       <c r="T39" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U39" s="2" t="inlineStr"/>
@@ -4219,7 +4261,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Uruguay vs Cape Verde</t>
+          <t>Uruguay vs Cape Verde Islands</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -4273,7 +4315,7 @@
       </c>
       <c r="T40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U40" s="2" t="inlineStr"/>
@@ -4363,7 +4405,7 @@
       </c>
       <c r="T41" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U41" s="2" t="inlineStr"/>
@@ -4453,7 +4495,7 @@
       </c>
       <c r="T42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U42" s="2" t="inlineStr"/>
@@ -4543,7 +4585,7 @@
       </c>
       <c r="T43" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U43" s="2" t="inlineStr"/>
@@ -4633,7 +4675,7 @@
       </c>
       <c r="T44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U44" s="2" t="inlineStr"/>
@@ -4723,7 +4765,7 @@
       </c>
       <c r="T45" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U45" s="2" t="inlineStr"/>
@@ -4813,7 +4855,7 @@
       </c>
       <c r="T46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U46" s="2" t="inlineStr"/>
@@ -4903,7 +4945,7 @@
       </c>
       <c r="T47" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U47" s="2" t="inlineStr"/>
@@ -4993,7 +5035,7 @@
       </c>
       <c r="T48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U48" s="2" t="inlineStr"/>
@@ -5029,7 +5071,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>Colombia vs DR Congo</t>
+          <t>Colombia vs Congo DR</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -5083,7 +5125,7 @@
       </c>
       <c r="T49" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U49" s="2" t="inlineStr"/>
@@ -5173,7 +5215,7 @@
       </c>
       <c r="T50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U50" s="2" t="inlineStr"/>
@@ -5209,7 +5251,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>Bosnia and Herzegovina vs Qatar</t>
+          <t>Bosnia &amp; Herzegovina vs Qatar</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -5263,7 +5305,7 @@
       </c>
       <c r="T51" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U51" s="2" t="inlineStr"/>
@@ -5353,7 +5395,7 @@
       </c>
       <c r="T52" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U52" s="2" t="inlineStr"/>
@@ -5443,7 +5485,7 @@
       </c>
       <c r="T53" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U53" s="2" t="inlineStr"/>
@@ -5479,7 +5521,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>Czech Republic vs Mexico</t>
+          <t>Czechia vs Mexico</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -5533,7 +5575,7 @@
       </c>
       <c r="T54" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U54" s="2" t="inlineStr"/>
@@ -5623,7 +5665,7 @@
       </c>
       <c r="T55" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U55" s="2" t="inlineStr"/>
@@ -5713,7 +5755,7 @@
       </c>
       <c r="T56" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U56" s="2" t="inlineStr"/>
@@ -5803,7 +5845,7 @@
       </c>
       <c r="T57" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U57" s="2" t="inlineStr"/>
@@ -5893,7 +5935,7 @@
       </c>
       <c r="T58" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U58" s="2" t="inlineStr"/>
@@ -5983,7 +6025,7 @@
       </c>
       <c r="T59" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U59" s="2" t="inlineStr"/>
@@ -6019,7 +6061,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>Turkey vs United States</t>
+          <t>Türkiye vs USA</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -6073,7 +6115,7 @@
       </c>
       <c r="T60" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U60" s="2" t="inlineStr"/>
@@ -6163,7 +6205,7 @@
       </c>
       <c r="T61" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U61" s="2" t="inlineStr"/>
@@ -6253,7 +6295,7 @@
       </c>
       <c r="T62" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U62" s="2" t="inlineStr"/>
@@ -6343,7 +6385,7 @@
       </c>
       <c r="T63" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U63" s="2" t="inlineStr"/>
@@ -6379,7 +6421,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>Cape Verde vs Saudi Arabia</t>
+          <t>Cape Verde Islands vs Saudi Arabia</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -6433,7 +6475,7 @@
       </c>
       <c r="T64" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U64" s="2" t="inlineStr"/>
@@ -6523,7 +6565,7 @@
       </c>
       <c r="T65" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U65" s="2" t="inlineStr"/>
@@ -6613,7 +6655,7 @@
       </c>
       <c r="T66" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U66" s="2" t="inlineStr"/>
@@ -6703,7 +6745,7 @@
       </c>
       <c r="T67" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U67" s="2" t="inlineStr"/>
@@ -6793,7 +6835,7 @@
       </c>
       <c r="T68" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U68" s="2" t="inlineStr"/>
@@ -6883,7 +6925,7 @@
       </c>
       <c r="T69" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U69" s="2" t="inlineStr"/>
@@ -6973,7 +7015,7 @@
       </c>
       <c r="T70" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U70" s="2" t="inlineStr"/>
@@ -7009,7 +7051,7 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>DR Congo vs Uzbekistan</t>
+          <t>Congo DR vs Uzbekistan</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -7063,7 +7105,7 @@
       </c>
       <c r="T71" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U71" s="2" t="inlineStr"/>
@@ -7153,7 +7195,7 @@
       </c>
       <c r="T72" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U72" s="2" t="inlineStr"/>
@@ -7243,7 +7285,7 @@
       </c>
       <c r="T73" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="U73" s="2" t="inlineStr"/>
@@ -7327,11 +7369,7 @@
           <t>否</t>
         </is>
       </c>
-      <c r="T74" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-10T00:00:00+08:00</t>
-        </is>
-      </c>
+      <c r="T74" s="2" t="inlineStr"/>
       <c r="U74" s="2" t="inlineStr"/>
       <c r="V74" s="2" t="inlineStr"/>
     </row>
@@ -7409,11 +7447,7 @@
           <t>否</t>
         </is>
       </c>
-      <c r="T75" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-10T00:00:00+08:00</t>
-        </is>
-      </c>
+      <c r="T75" s="2" t="inlineStr"/>
       <c r="U75" s="2" t="inlineStr"/>
       <c r="V75" s="2" t="inlineStr"/>
     </row>
@@ -7491,11 +7525,7 @@
           <t>否</t>
         </is>
       </c>
-      <c r="T76" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-10T00:00:00+08:00</t>
-        </is>
-      </c>
+      <c r="T76" s="2" t="inlineStr"/>
       <c r="U76" s="2" t="inlineStr"/>
       <c r="V76" s="2" t="inlineStr"/>
     </row>
@@ -7573,11 +7603,7 @@
           <t>否</t>
         </is>
       </c>
-      <c r="T77" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-10T00:00:00+08:00</t>
-        </is>
-      </c>
+      <c r="T77" s="2" t="inlineStr"/>
       <c r="U77" s="2" t="inlineStr"/>
       <c r="V77" s="2" t="inlineStr"/>
     </row>
@@ -7655,11 +7681,7 @@
           <t>否</t>
         </is>
       </c>
-      <c r="T78" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-10T00:00:00+08:00</t>
-        </is>
-      </c>
+      <c r="T78" s="2" t="inlineStr"/>
       <c r="U78" s="2" t="inlineStr"/>
       <c r="V78" s="2" t="inlineStr"/>
     </row>
@@ -7737,11 +7759,7 @@
           <t>否</t>
         </is>
       </c>
-      <c r="T79" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-10T00:00:00+08:00</t>
-        </is>
-      </c>
+      <c r="T79" s="2" t="inlineStr"/>
       <c r="U79" s="2" t="inlineStr"/>
       <c r="V79" s="2" t="inlineStr"/>
     </row>
@@ -7819,11 +7837,7 @@
           <t>否</t>
         </is>
       </c>
-      <c r="T80" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-10T00:00:00+08:00</t>
-        </is>
-      </c>
+      <c r="T80" s="2" t="inlineStr"/>
       <c r="U80" s="2" t="inlineStr"/>
       <c r="V80" s="2" t="inlineStr"/>
     </row>
@@ -7901,11 +7915,7 @@
           <t>否</t>
         </is>
       </c>
-      <c r="T81" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-10T00:00:00+08:00</t>
-        </is>
-      </c>
+      <c r="T81" s="2" t="inlineStr"/>
       <c r="U81" s="2" t="inlineStr"/>
       <c r="V81" s="2" t="inlineStr"/>
     </row>
@@ -7983,11 +7993,7 @@
           <t>否</t>
         </is>
       </c>
-      <c r="T82" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-10T00:00:00+08:00</t>
-        </is>
-      </c>
+      <c r="T82" s="2" t="inlineStr"/>
       <c r="U82" s="2" t="inlineStr"/>
       <c r="V82" s="2" t="inlineStr"/>
     </row>
@@ -8065,11 +8071,7 @@
           <t>否</t>
         </is>
       </c>
-      <c r="T83" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-10T00:00:00+08:00</t>
-        </is>
-      </c>
+      <c r="T83" s="2" t="inlineStr"/>
       <c r="U83" s="2" t="inlineStr"/>
       <c r="V83" s="2" t="inlineStr"/>
     </row>
@@ -8147,11 +8149,7 @@
           <t>否</t>
         </is>
       </c>
-      <c r="T84" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-10T00:00:00+08:00</t>
-        </is>
-      </c>
+      <c r="T84" s="2" t="inlineStr"/>
       <c r="U84" s="2" t="inlineStr"/>
       <c r="V84" s="2" t="inlineStr"/>
     </row>
@@ -8229,11 +8227,7 @@
           <t>否</t>
         </is>
       </c>
-      <c r="T85" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-10T00:00:00+08:00</t>
-        </is>
-      </c>
+      <c r="T85" s="2" t="inlineStr"/>
       <c r="U85" s="2" t="inlineStr"/>
       <c r="V85" s="2" t="inlineStr"/>
     </row>
@@ -8311,11 +8305,7 @@
           <t>否</t>
         </is>
       </c>
-      <c r="T86" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-10T00:00:00+08:00</t>
-        </is>
-      </c>
+      <c r="T86" s="2" t="inlineStr"/>
       <c r="U86" s="2" t="inlineStr"/>
       <c r="V86" s="2" t="inlineStr"/>
     </row>
@@ -8393,11 +8383,7 @@
           <t>否</t>
         </is>
       </c>
-      <c r="T87" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-10T00:00:00+08:00</t>
-        </is>
-      </c>
+      <c r="T87" s="2" t="inlineStr"/>
       <c r="U87" s="2" t="inlineStr"/>
       <c r="V87" s="2" t="inlineStr"/>
     </row>
@@ -8475,11 +8461,7 @@
           <t>否</t>
         </is>
       </c>
-      <c r="T88" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-10T00:00:00+08:00</t>
-        </is>
-      </c>
+      <c r="T88" s="2" t="inlineStr"/>
       <c r="U88" s="2" t="inlineStr"/>
       <c r="V88" s="2" t="inlineStr"/>
     </row>
@@ -8557,11 +8539,7 @@
           <t>否</t>
         </is>
       </c>
-      <c r="T89" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-10T00:00:00+08:00</t>
-        </is>
-      </c>
+      <c r="T89" s="2" t="inlineStr"/>
       <c r="U89" s="2" t="inlineStr"/>
       <c r="V89" s="2" t="inlineStr"/>
     </row>
@@ -8639,11 +8617,7 @@
           <t>否</t>
         </is>
       </c>
-      <c r="T90" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-10T00:00:00+08:00</t>
-        </is>
-      </c>
+      <c r="T90" s="2" t="inlineStr"/>
       <c r="U90" s="2" t="inlineStr"/>
       <c r="V90" s="2" t="inlineStr"/>
     </row>
@@ -8721,11 +8695,7 @@
           <t>否</t>
         </is>
       </c>
-      <c r="T91" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-10T00:00:00+08:00</t>
-        </is>
-      </c>
+      <c r="T91" s="2" t="inlineStr"/>
       <c r="U91" s="2" t="inlineStr"/>
       <c r="V91" s="2" t="inlineStr"/>
     </row>
@@ -8803,11 +8773,7 @@
           <t>否</t>
         </is>
       </c>
-      <c r="T92" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-10T00:00:00+08:00</t>
-        </is>
-      </c>
+      <c r="T92" s="2" t="inlineStr"/>
       <c r="U92" s="2" t="inlineStr"/>
       <c r="V92" s="2" t="inlineStr"/>
     </row>
@@ -8885,11 +8851,7 @@
           <t>否</t>
         </is>
       </c>
-      <c r="T93" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-10T00:00:00+08:00</t>
-        </is>
-      </c>
+      <c r="T93" s="2" t="inlineStr"/>
       <c r="U93" s="2" t="inlineStr"/>
       <c r="V93" s="2" t="inlineStr"/>
     </row>
@@ -8967,11 +8929,7 @@
           <t>否</t>
         </is>
       </c>
-      <c r="T94" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-10T00:00:00+08:00</t>
-        </is>
-      </c>
+      <c r="T94" s="2" t="inlineStr"/>
       <c r="U94" s="2" t="inlineStr"/>
       <c r="V94" s="2" t="inlineStr"/>
     </row>
@@ -9049,11 +9007,7 @@
           <t>否</t>
         </is>
       </c>
-      <c r="T95" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-10T00:00:00+08:00</t>
-        </is>
-      </c>
+      <c r="T95" s="2" t="inlineStr"/>
       <c r="U95" s="2" t="inlineStr"/>
       <c r="V95" s="2" t="inlineStr"/>
     </row>
@@ -9131,11 +9085,7 @@
           <t>否</t>
         </is>
       </c>
-      <c r="T96" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-10T00:00:00+08:00</t>
-        </is>
-      </c>
+      <c r="T96" s="2" t="inlineStr"/>
       <c r="U96" s="2" t="inlineStr"/>
       <c r="V96" s="2" t="inlineStr"/>
     </row>
@@ -9213,11 +9163,7 @@
           <t>否</t>
         </is>
       </c>
-      <c r="T97" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-10T00:00:00+08:00</t>
-        </is>
-      </c>
+      <c r="T97" s="2" t="inlineStr"/>
       <c r="U97" s="2" t="inlineStr"/>
       <c r="V97" s="2" t="inlineStr"/>
     </row>
@@ -9295,11 +9241,7 @@
           <t>否</t>
         </is>
       </c>
-      <c r="T98" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-10T00:00:00+08:00</t>
-        </is>
-      </c>
+      <c r="T98" s="2" t="inlineStr"/>
       <c r="U98" s="2" t="inlineStr"/>
       <c r="V98" s="2" t="inlineStr"/>
     </row>
@@ -9377,11 +9319,7 @@
           <t>否</t>
         </is>
       </c>
-      <c r="T99" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-10T00:00:00+08:00</t>
-        </is>
-      </c>
+      <c r="T99" s="2" t="inlineStr"/>
       <c r="U99" s="2" t="inlineStr"/>
       <c r="V99" s="2" t="inlineStr"/>
     </row>
@@ -9459,11 +9397,7 @@
           <t>否</t>
         </is>
       </c>
-      <c r="T100" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-10T00:00:00+08:00</t>
-        </is>
-      </c>
+      <c r="T100" s="2" t="inlineStr"/>
       <c r="U100" s="2" t="inlineStr"/>
       <c r="V100" s="2" t="inlineStr"/>
     </row>
@@ -9541,11 +9475,7 @@
           <t>否</t>
         </is>
       </c>
-      <c r="T101" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-10T00:00:00+08:00</t>
-        </is>
-      </c>
+      <c r="T101" s="2" t="inlineStr"/>
       <c r="U101" s="2" t="inlineStr"/>
       <c r="V101" s="2" t="inlineStr"/>
     </row>
@@ -9623,11 +9553,7 @@
           <t>否</t>
         </is>
       </c>
-      <c r="T102" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-10T00:00:00+08:00</t>
-        </is>
-      </c>
+      <c r="T102" s="2" t="inlineStr"/>
       <c r="U102" s="2" t="inlineStr"/>
       <c r="V102" s="2" t="inlineStr"/>
     </row>
@@ -9705,11 +9631,7 @@
           <t>否</t>
         </is>
       </c>
-      <c r="T103" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-10T00:00:00+08:00</t>
-        </is>
-      </c>
+      <c r="T103" s="2" t="inlineStr"/>
       <c r="U103" s="2" t="inlineStr"/>
       <c r="V103" s="2" t="inlineStr"/>
     </row>
@@ -9787,11 +9709,7 @@
           <t>否</t>
         </is>
       </c>
-      <c r="T104" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-10T00:00:00+08:00</t>
-        </is>
-      </c>
+      <c r="T104" s="2" t="inlineStr"/>
       <c r="U104" s="2" t="inlineStr"/>
       <c r="V104" s="2" t="inlineStr"/>
     </row>
@@ -9869,11 +9787,7 @@
           <t>否</t>
         </is>
       </c>
-      <c r="T105" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-10T00:00:00+08:00</t>
-        </is>
-      </c>
+      <c r="T105" s="2" t="inlineStr"/>
       <c r="U105" s="2" t="inlineStr"/>
       <c r="V105" s="2" t="inlineStr"/>
     </row>
@@ -10070,14 +9984,14 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Czech Republic</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F2" s="2" t="n">
         <v>0</v>
@@ -10086,16 +10000,16 @@
         <v>0</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L2" s="2" t="n">
         <v>0</v>
@@ -10117,14 +10031,14 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>South Korea</t>
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>0</v>
@@ -10133,16 +10047,16 @@
         <v>0</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L3" s="2" t="n">
         <v>0</v>
@@ -10164,11 +10078,11 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Czech Republic</t>
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4" s="2" t="n">
         <v>0</v>
@@ -10177,16 +10091,16 @@
         <v>0</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="K4" s="2" t="n">
         <v>0</v>
@@ -10211,11 +10125,11 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>South Korea</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>0</v>
@@ -10224,16 +10138,16 @@
         <v>0</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H5" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="K5" s="2" t="n">
         <v>0</v>
@@ -10262,28 +10176,28 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E6" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>0</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L6" s="2" t="n">
         <v>0</v>
@@ -10309,28 +10223,28 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>0</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J7" s="2" t="n">
         <v>0</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L7" s="2" t="n">
         <v>0</v>
@@ -10634,14 +10548,14 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F14" s="2" t="n">
         <v>0</v>
@@ -10650,16 +10564,16 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J14" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K14" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L14" s="2" t="n">
         <v>0</v>
@@ -10681,7 +10595,7 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Paraguay</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="D15" s="2" t="n">
@@ -10775,11 +10689,11 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Paraguay</t>
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E17" s="2" t="n">
         <v>0</v>
@@ -10788,16 +10702,16 @@
         <v>0</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J17" s="2" t="n">
-        <v>0</v>
+        <v>-3</v>
       </c>
       <c r="K17" s="2" t="n">
         <v>0</v>
@@ -12335,7 +12249,7 @@
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
     <col width="9" customWidth="1" min="5" max="5"/>
     <col width="9" customWidth="1" min="6" max="6"/>
@@ -12647,12 +12561,12 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>H</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="D10" s="6" t="n">
@@ -12679,12 +12593,12 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>F</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="D11" s="6" t="n">
@@ -12711,12 +12625,12 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="D12" s="6" t="n">
@@ -12743,22 +12657,22 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>Czech Republic</t>
         </is>
       </c>
       <c r="D13" s="6" t="n">
         <v>0</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="F13" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G13" s="6" t="n">
         <v>0</v>
@@ -14842,12 +14756,12 @@
     <col width="9" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="39" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
     <col width="9" customWidth="1" min="5" max="5"/>
     <col width="9" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
     <col width="9" customWidth="1" min="8" max="8"/>
-    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
     <col width="37" customWidth="1" min="10" max="10"/>
     <col width="9" customWidth="1" min="11" max="11"/>
   </cols>
@@ -14930,16 +14844,28 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr"/>
+          <t>已结束</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>90+8</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
       <c r="H2" s="2" t="inlineStr"/>
-      <c r="I2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12 周五 02:00 (Asia/Shanghai)</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr"/>
@@ -14960,21 +14886,33 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>South Korea vs Czech Republic</t>
+          <t>South Korea vs Czechia</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr"/>
-      <c r="G3" s="2" t="inlineStr"/>
+          <t>已结束</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>90+7</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
       <c r="H3" s="2" t="inlineStr"/>
-      <c r="I3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12 周五 09:00 (Asia/Shanghai)</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr"/>
@@ -14995,21 +14933,29 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Canada vs Bosnia and Herzegovina</t>
+          <t>Canada vs Bosnia &amp; Herzegovina</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr"/>
-      <c r="G4" s="2" t="inlineStr"/>
+          <t>已结束</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>90+6</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
       <c r="H4" s="2" t="inlineStr"/>
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13 周六 02:00 (Asia/Shanghai)</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr"/>
@@ -15030,21 +14976,31 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>United States vs Paraguay</t>
+          <t>USA vs Paraguay</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr"/>
-      <c r="G5" s="2" t="inlineStr"/>
+          <t>已结束</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>90</v>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>4-1</t>
+        </is>
+      </c>
       <c r="H5" s="2" t="inlineStr"/>
-      <c r="I5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13 周六 08:00 (Asia/Shanghai)</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr"/>
@@ -15170,7 +15126,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Australia vs Turkey</t>
+          <t>Australia vs Türkiye</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -15345,7 +15301,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Spain vs Cape Verde</t>
+          <t>Spain vs Cape Verde Islands</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -15625,7 +15581,7 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Portugal vs DR Congo</t>
+          <t>Portugal vs Congo DR</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -15765,7 +15721,7 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Czech Republic vs South Africa</t>
+          <t>Czechia vs South Africa</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -15800,7 +15756,7 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Switzerland vs Bosnia and Herzegovina</t>
+          <t>Switzerland vs Bosnia &amp; Herzegovina</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -15905,7 +15861,7 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>United States vs Australia</t>
+          <t>USA vs Australia</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -16010,7 +15966,7 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Turkey vs Paraguay</t>
+          <t>Türkiye vs Paraguay</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -16255,7 +16211,7 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Uruguay vs Cape Verde</t>
+          <t>Uruguay vs Cape Verde Islands</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
@@ -16570,7 +16526,7 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>Colombia vs DR Congo</t>
+          <t>Colombia vs Congo DR</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
@@ -16640,7 +16596,7 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>Bosnia and Herzegovina vs Qatar</t>
+          <t>Bosnia &amp; Herzegovina vs Qatar</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
@@ -16745,7 +16701,7 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Czech Republic vs Mexico</t>
+          <t>Czechia vs Mexico</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
@@ -16955,7 +16911,7 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Turkey vs United States</t>
+          <t>Türkiye vs USA</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
@@ -17095,7 +17051,7 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Cape Verde vs Saudi Arabia</t>
+          <t>Cape Verde Islands vs Saudi Arabia</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
@@ -17340,7 +17296,7 @@
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>DR Congo vs Uzbekistan</t>
+          <t>Congo DR vs Uzbekistan</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
@@ -18587,7 +18543,7 @@
       </c>
       <c r="B2" s="8" t="inlineStr">
         <is>
-          <t>2026-06-10T13:34:44Z</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
     </row>
@@ -18599,7 +18555,7 @@
       </c>
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00+08:00</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
     </row>
@@ -18611,7 +18567,7 @@
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>2026-06-10T13:34:44Z</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
     </row>
@@ -18623,7 +18579,7 @@
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>2026-06-10T13:34:44Z</t>
+          <t>2026-06-13T08:50:26Z</t>
         </is>
       </c>
     </row>

</xml_diff>